<commit_message>
Add bulk select + bulk price change for products and rooms
Many products/rooms were priced identically then set wrong all at once,
so fixing them one by one was tedious. Both management pages now have a
checkbox per row (+ select-all) and a bulk action bar for setting a new
price, hiding/showing (products) or opening/closing (rooms), and deleting
- reusing the same safe delete-or-hide/close fallback as the single-item
delete buttons, so a bulk delete across items with and without order/
booking history does the right thing for each one individually.

_delete_product_or_hide and _delete_room_or_close are extracted from the
existing single-delete routes so both the single and bulk paths share one
implementation.

Verified live in a real browser (bulk select, price applied correctly,
untouched rows unaffected) plus 4 new CRUD test cases (SP-08/09, PH-07/08)
in the Test case/ suite - 45/45 passing.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test case/test_cases.xlsx
+++ b/Test case/test_cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -851,32 +851,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PH-01</t>
+          <t>SP-08</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Phòng</t>
+          <t>Sản phẩm</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Thêm phòng mới</t>
+          <t>Đổi giá hàng loạt nhiều sản phẩm</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Admin điền form và lưu phòng mới</t>
+          <t>Admin chọn nhiều sản phẩm cùng lúc rồi nhập một giá mới, áp dụng cho tất cả</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Phòng xuất hiện trong danh sách quản lý phòng</t>
+          <t>Tất cả sản phẩm được chọn đổi thành đúng giá mới, sản phẩm không được chọn giữ nguyên giá cũ</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -886,12 +886,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>5 -&gt; 6</t>
+          <t>A=18000.0 B=18000.0 untouched=33333.0</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -901,32 +901,32 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PH-02</t>
+          <t>SP-09</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Phòng</t>
+          <t>Sản phẩm</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Sửa phòng</t>
+          <t>Xóa hàng loạt nhiều sản phẩm</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Admin đổi tên, giá, sức chứa của một phòng có sẵn</t>
+          <t>Admin chọn nhiều sản phẩm (một sản phẩm chưa từng bán, một sản phẩm đã có đơn hàng) rồi xóa cùng lúc</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Thông tin phòng được cập nhật đúng như đã sửa</t>
+          <t>Sản phẩm chưa từng bán bị xóa hẳn; sản phẩm đã có đơn hàng chỉ bị ẩn - giống hệt quy tắc xóa từng cái một</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -934,10 +934,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>A đã xóa hẳn=True, B đã có đơn nên chỉ ẩn=True</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -947,7 +951,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PH-03</t>
+          <t>PH-01</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -957,22 +961,22 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Bật/tắt trạng thái phòng trống</t>
+          <t>Thêm phòng mới</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Admin bấm nút đổi trạng thái mở/đóng phòng</t>
+          <t>Admin điền form và lưu phòng mới</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái available đảo ngược đúng</t>
+          <t>Phòng xuất hiện trong danh sách quản lý phòng</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -980,10 +984,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>5 -&gt; 6</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -993,7 +1001,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PH-04</t>
+          <t>PH-02</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1003,22 +1011,22 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Xóa phòng chưa từng có lịch đặt</t>
+          <t>Sửa phòng</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Admin xóa một phòng chưa từng được đặt</t>
+          <t>Admin đổi tên, giá, sức chứa của một phòng có sẵn</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Phòng bị xóa hẳn khỏi cơ sở dữ liệu</t>
+          <t>Thông tin phòng được cập nhật đúng như đã sửa</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1029,7 +1037,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1047,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PH-05</t>
+          <t>PH-03</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1049,22 +1057,22 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Xóa phòng đã có lịch đặt</t>
+          <t>Bật/tắt trạng thái phòng trống</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Admin xóa một phòng đã từng có người đặt (RoomBooking)</t>
+          <t>Admin bấm nút đổi trạng thái mở/đóng phòng</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Không xóa hẳn (vì phá vỡ lịch sử đặt phòng) - tự động đóng phòng, lịch sử vẫn giữ nguyên</t>
+          <t>Trạng thái available đảo ngược đúng</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1072,14 +1080,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>phòng vẫn còn nhưng available=False</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1093,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PH-06</t>
+          <t>PH-04</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1099,22 +1103,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật trạng thái đặt phòng</t>
+          <t>Xóa phòng chưa từng có lịch đặt</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Admin đổi trạng thái một lượt đặt phòng (chờ/xác nhận/hủy)</t>
+          <t>Admin xóa một phòng chưa từng được đặt</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái đặt phòng được cập nhật đúng</t>
+          <t>Phòng bị xóa hẳn khỏi cơ sở dữ liệu</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1125,7 +1129,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1135,32 +1139,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>DH-01</t>
+          <t>PH-05</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng</t>
+          <t>Phòng</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Tạo đơn tại quầy (POS)</t>
+          <t>Xóa phòng đã có lịch đặt</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Admin chọn món và tạo đơn ngay tại quầy bán hàng</t>
+          <t>Admin xóa một phòng đã từng có người đặt (RoomBooking)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng mới được tạo, tồn kho sản phẩm bị trừ đúng số lượng</t>
+          <t>Không xóa hẳn (vì phá vỡ lịch sử đặt phòng) - tự động đóng phòng, lịch sử vẫn giữ nguyên</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1170,12 +1174,12 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>đơn 5-&gt;6, tồn kho 47-&gt;46</t>
+          <t>phòng vẫn còn nhưng available=False</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1185,17 +1189,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>DH-02</t>
+          <t>PH-06</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng</t>
+          <t>Phòng</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật trạng thái đơn hàng</t>
+          <t>Cập nhật trạng thái đặt phòng</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1205,12 +1209,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Admin đổi trạng thái đơn từ "còn nợ" sang "hoàn thành"</t>
+          <t>Admin đổi trạng thái một lượt đặt phòng (chờ/xác nhận/hủy)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái đơn hàng được cập nhật đúng</t>
+          <t>Trạng thái đặt phòng được cập nhật đúng</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1221,7 +1225,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1231,32 +1235,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>DH-03</t>
+          <t>PH-07</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng</t>
+          <t>Phòng</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Xóa đơn hàng - Super Admin</t>
+          <t>Đổi giá hàng loạt nhiều phòng</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Super Admin xóa một đơn hàng test</t>
+          <t>Admin chọn nhiều phòng cùng lúc rồi nhập một giá thuê mới, áp dụng cho tất cả</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng và các dòng sản phẩm trong đơn bị xóa hẳn</t>
+          <t>Tất cả phòng được chọn đổi thành đúng giá mới, phòng không được chọn giữ nguyên giá cũ</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1264,10 +1268,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>A=1800000.0 B=1800000.0 untouched=3000000.0</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1277,17 +1285,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>DH-04</t>
+          <t>PH-08</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng</t>
+          <t>Phòng</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Xóa đơn hàng - Admin thường (phải bị chặn)</t>
+          <t>Xóa hàng loạt nhiều phòng</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1297,12 +1305,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản admin thường (không phải Super Admin) cố xóa một đơn hàng</t>
+          <t>Admin chọn nhiều phòng (một phòng chưa từng có lịch đặt, một phòng đã có lịch đặt) rồi xóa cùng lúc</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Bị từ chối, đơn hàng vẫn còn nguyên - chỉ Super Admin mới được xóa</t>
+          <t>Phòng chưa từng có lịch đặt bị xóa hẳn; phòng đã có lịch đặt chỉ bị đóng - giống hệt quy tắc xóa từng cái một</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1312,12 +1320,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>còn tồn tại=True thông báo chặn=True</t>
+          <t>A đã xóa hẳn=True, B đã có lịch nên chỉ đóng=True</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1335,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>DH-05</t>
+          <t>DH-01</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1337,7 +1345,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Khách đặt hàng qua giỏ hàng</t>
+          <t>Tạo đơn tại quầy (POS)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1347,12 +1355,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Khách thêm sản phẩm vào giỏ rồi đặt hàng (checkout)</t>
+          <t>Admin chọn món và tạo đơn ngay tại quầy bán hàng</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Đơn hàng mới được tạo với đúng tên/số điện thoại khách đã nhập</t>
+          <t>Đơn hàng mới được tạo, tồn kho sản phẩm bị trừ đúng số lượng</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1362,12 +1370,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>4 -&gt; 5</t>
+          <t>đơn 6-&gt;7, tồn kho 49-&gt;48</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1377,32 +1385,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>GH-01</t>
+          <t>DH-02</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Thêm vào giỏ hàng</t>
+          <t>Cập nhật trạng thái đơn hàng</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Khách thêm một sản phẩm vào giỏ hàng</t>
+          <t>Admin đổi trạng thái đơn từ "còn nợ" sang "hoàn thành"</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Sản phẩm xuất hiện trong giỏ với đúng số lượng</t>
+          <t>Trạng thái đơn hàng được cập nhật đúng</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1413,7 +1421,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1423,32 +1431,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>GH-02</t>
+          <t>DH-03</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật số lượng trong giỏ</t>
+          <t>Xóa đơn hàng - Super Admin</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Khách đổi số lượng một sản phẩm đang có trong giỏ</t>
+          <t>Tài khoản Super Admin xóa một đơn hàng test</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Số lượng trong giỏ được cập nhật đúng</t>
+          <t>Đơn hàng và các dòng sản phẩm trong đơn bị xóa hẳn</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1459,7 +1467,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1469,17 +1477,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>GH-03</t>
+          <t>DH-04</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Xóa một món khỏi giỏ</t>
+          <t>Xóa đơn hàng - Admin thường (phải bị chặn)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1489,12 +1497,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Khách xóa một sản phẩm khỏi giỏ hàng</t>
+          <t>Tài khoản admin thường (không phải Super Admin) cố xóa một đơn hàng</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Sản phẩm biến mất khỏi giỏ hàng</t>
+          <t>Bị từ chối, đơn hàng vẫn còn nguyên - chỉ Super Admin mới được xóa</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1502,10 +1510,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>còn tồn tại=True thông báo chặn=True</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1515,32 +1527,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>GH-04</t>
+          <t>DH-05</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Xóa nhiều món cùng lúc</t>
+          <t>Khách đặt hàng qua giỏ hàng</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Khách tick chọn nhiều sản phẩm rồi xóa cùng lúc</t>
+          <t>Khách thêm sản phẩm vào giỏ rồi đặt hàng (checkout)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Chỉ những sản phẩm được chọn bị xóa, các món khác vẫn còn</t>
+          <t>Đơn hàng mới được tạo với đúng tên/số điện thoại khách đã nhập</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1550,12 +1562,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>gone=True kept=True</t>
+          <t>5 -&gt; 6</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1565,32 +1577,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>CN-01</t>
+          <t>GH-01</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Công nợ</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Thanh toán một đơn nợ</t>
+          <t>Thêm vào giỏ hàng</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Super Admin xác nhận một đơn còn nợ đã được trả</t>
+          <t>Khách thêm một sản phẩm vào giỏ hàng</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái đơn chuyển thành hoàn thành</t>
+          <t>Sản phẩm xuất hiện trong giỏ với đúng số lượng</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -1601,7 +1613,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1611,17 +1623,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>CN-02</t>
+          <t>GH-02</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Công nợ</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Thanh toán nhiều đơn nợ cùng lúc</t>
+          <t>Cập nhật số lượng trong giỏ</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1631,12 +1643,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Super Admin chọn nhiều đơn nợ và xác nhận trả cùng lúc</t>
+          <t>Khách đổi số lượng một sản phẩm đang có trong giỏ</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Tất cả các đơn được chọn chuyển thành hoàn thành</t>
+          <t>Số lượng trong giỏ được cập nhật đúng</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1647,7 +1659,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1657,32 +1669,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>TK-01</t>
+          <t>GH-03</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Thêm tài khoản admin mới</t>
+          <t>Xóa một món khỏi giỏ</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Super Admin tạo một tài khoản admin mới</t>
+          <t>Khách xóa một sản phẩm khỏi giỏ hàng</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản mới xuất hiện trong danh sách, đăng nhập được</t>
+          <t>Sản phẩm biến mất khỏi giỏ hàng</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -1690,14 +1702,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>2 -&gt; 3</t>
-        </is>
-      </c>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1707,32 +1715,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TK-02</t>
+          <t>GH-04</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Đổi vai trò admin</t>
+          <t>Xóa nhiều món cùng lúc</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đổi vai trò một tài khoản admin thành super_admin</t>
+          <t>Khách tick chọn nhiều sản phẩm rồi xóa cùng lúc</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Vai trò được cập nhật đúng</t>
+          <t>Chỉ những sản phẩm được chọn bị xóa, các món khác vẫn còn</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -1740,10 +1748,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>gone=True kept=True</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1753,17 +1765,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>TK-03</t>
+          <t>CN-01</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Công nợ</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Đặt lại mật khẩu admin</t>
+          <t>Thanh toán một đơn nợ</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1773,12 +1785,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đặt mật khẩu mới cho một tài khoản admin khác</t>
+          <t>Super Admin xác nhận một đơn còn nợ đã được trả</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản đó đăng nhập được bằng mật khẩu mới</t>
+          <t>Trạng thái đơn chuyển thành hoàn thành</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -1789,7 +1801,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1799,17 +1811,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>TK-04</t>
+          <t>CN-02</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Công nợ</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Đặt lại mật khẩu khách hàng</t>
+          <t>Thanh toán nhiều đơn nợ cùng lúc</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1819,12 +1831,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đặt mật khẩu mới cho một tài khoản khách hàng</t>
+          <t>Super Admin chọn nhiều đơn nợ và xác nhận trả cùng lúc</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản khách hàng đăng nhập được bằng mật khẩu mới</t>
+          <t>Tất cả các đơn được chọn chuyển thành hoàn thành</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1835,7 +1847,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1857,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>TK-05</t>
+          <t>TK-01</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1855,22 +1867,22 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Xóa tài khoản admin</t>
+          <t>Thêm tài khoản admin mới</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Super Admin xóa một tài khoản admin (không phải Super Admin cuối cùng)</t>
+          <t>Super Admin tạo một tài khoản admin mới</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản bị xóa hẳn, không đăng nhập được nữa</t>
+          <t>Tài khoản mới xuất hiện trong danh sách, đăng nhập được</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -1878,10 +1890,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>2 -&gt; 3</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1907,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>TK-06</t>
+          <t>TK-02</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1901,22 +1917,22 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Không cho xóa Super Admin cuối cùng</t>
+          <t>Đổi vai trò admin</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Super Admin cố xóa chính Super Admin cuối cùng còn lại trong hệ thống</t>
+          <t>Super Admin đổi vai trò một tài khoản admin thành super_admin</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Bị từ chối, luôn còn ít nhất một Super Admin</t>
+          <t>Vai trò được cập nhật đúng</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -1924,14 +1940,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>còn tồn tại=True</t>
-        </is>
-      </c>
+      <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1953,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>TK-07</t>
+          <t>TK-03</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1951,7 +1963,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Bật/tắt quyền Manager</t>
+          <t>Đặt lại mật khẩu admin</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1961,12 +1973,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Super Admin cấp rồi thu hồi quyền Manager cho một khách hàng</t>
+          <t>Super Admin đặt mật khẩu mới cho một tài khoản admin khác</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Vai trò khách hàng đổi qua lại đúng giữa customer và manager</t>
+          <t>Tài khoản đó đăng nhập được bằng mật khẩu mới</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1974,14 +1986,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>promoted=True back=True</t>
-        </is>
-      </c>
+      <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1999,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>TK-08</t>
+          <t>TK-04</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2001,22 +2009,22 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Đăng ký tài khoản khách hàng</t>
+          <t>Đặt lại mật khẩu khách hàng</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Khách tự đăng ký tài khoản mới trên trang web</t>
+          <t>Super Admin đặt mật khẩu mới cho một tài khoản khách hàng</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản khách hàng mới được tạo, đăng nhập được ngay</t>
+          <t>Tài khoản khách hàng đăng nhập được bằng mật khẩu mới</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -2024,14 +2032,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>0 -&gt; 1</t>
-        </is>
-      </c>
+      <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2041,32 +2045,32 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>XT-01</t>
+          <t>TK-05</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập admin đúng mật khẩu</t>
+          <t>Xóa tài khoản admin</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập với tài khoản/mật khẩu admin đúng</t>
+          <t>Super Admin xóa một tài khoản admin (không phải Super Admin cuối cùng)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập thành công, vào được trang quản trị</t>
+          <t>Tài khoản bị xóa hẳn, không đăng nhập được nữa</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -2077,7 +2081,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2087,32 +2091,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>XT-02</t>
+          <t>TK-06</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập admin sai mật khẩu</t>
+          <t>Không cho xóa Super Admin cuối cùng</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập với mật khẩu sai</t>
+          <t>Super Admin cố xóa chính Super Admin cuối cùng còn lại trong hệ thống</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Bị từ chối, không vào được trang quản trị</t>
+          <t>Bị từ chối, luôn còn ít nhất một Super Admin</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2122,12 +2126,12 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302</t>
+          <t>còn tồn tại=True</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2137,17 +2141,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>XT-03</t>
+          <t>TK-07</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Admin tự đổi mật khẩu</t>
+          <t>Bật/tắt quyền Manager</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2157,12 +2161,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Admin đang đăng nhập tự đổi mật khẩu của chính mình</t>
+          <t>Super Admin cấp rồi thu hồi quyền Manager cho một khách hàng</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập lại bằng mật khẩu mới thành công</t>
+          <t>Vai trò khách hàng đổi qua lại đúng giữa customer và manager</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -2170,10 +2174,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>promoted=True back=True</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2183,32 +2191,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>XT-04</t>
+          <t>TK-08</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập khách hàng</t>
+          <t>Đăng ký tài khoản khách hàng</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Khách đăng nhập bằng tài khoản đã đăng ký</t>
+          <t>Khách tự đăng ký tài khoản mới trên trang web</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập thành công</t>
+          <t>Tài khoản khách hàng mới được tạo, đăng nhập được ngay</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -2218,12 +2226,12 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302</t>
+          <t>0 -&gt; 1</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2241,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>XT-05</t>
+          <t>XT-01</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2243,7 +2251,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Đăng xuất khách hàng</t>
+          <t>Đăng nhập admin đúng mật khẩu</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2253,12 +2261,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Khách đã đăng nhập bấm đăng xuất</t>
+          <t>Đăng nhập với tài khoản/mật khẩu admin đúng</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Phiên đăng nhập kết thúc</t>
+          <t>Đăng nhập thành công, vào được trang quản trị</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2269,7 +2277,7 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2279,32 +2287,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>QR-01</t>
+          <t>XT-02</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>QR / Thanh toán</t>
+          <t>Xác thực</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Tạo mã QR tuỳ ý</t>
+          <t>Đăng nhập admin sai mật khẩu</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Admin tạo một mã QR từ nội dung bất kỳ</t>
+          <t>Đăng nhập với mật khẩu sai</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Ảnh mã QR được sinh ra thành công</t>
+          <t>Bị từ chối, không vào được trang quản trị</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2312,10 +2320,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 302</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2325,32 +2337,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>QR-02</t>
+          <t>XT-03</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>QR / Thanh toán</t>
+          <t>Xác thực</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Tạo mã QR chuyển khoản ngân hàng</t>
+          <t>Admin tự đổi mật khẩu</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Admin tạo mã QR chuyển khoản với số tiền và nội dung</t>
+          <t>Admin đang đăng nhập tự đổi mật khẩu của chính mình</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Ảnh mã QR VietQR được sinh ra thành công</t>
+          <t>Đăng nhập lại bằng mật khẩu mới thành công</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2361,7 +2373,7 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2371,32 +2383,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>QR-03</t>
+          <t>XT-04</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>QR / Thanh toán</t>
+          <t>Xác thực</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Đặt tài khoản nhận tiền mặc định</t>
+          <t>Đăng nhập khách hàng</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đặt một tài khoản ngân hàng làm tài khoản nhận tiền mặc định của quán</t>
+          <t>Khách đăng nhập bằng tài khoản đã đăng ký</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Cấu hình được lưu lại, dùng cho mọi mã QR sau này</t>
+          <t>Đăng nhập thành công</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -2411,7 +2423,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:11</t>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>
@@ -2421,47 +2433,235 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
+          <t>XT-05</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Xác thực</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Đăng xuất khách hàng</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Khách đã đăng nhập bấm đăng xuất</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Phiên đăng nhập kết thúc</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>QR-01</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>QR / Thanh toán</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Tạo mã QR tuỳ ý</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Thêm</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Admin tạo một mã QR từ nội dung bất kỳ</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh mã QR được sinh ra thành công</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>QR-02</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>QR / Thanh toán</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Tạo mã QR chuyển khoản ngân hàng</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Thêm</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Admin tạo mã QR chuyển khoản với số tiền và nội dung</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh mã QR VietQR được sinh ra thành công</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>QR-03</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>QR / Thanh toán</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Đặt tài khoản nhận tiền mặc định</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Sửa</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Super Admin đặt một tài khoản ngân hàng làm tài khoản nhận tiền mặc định của quán</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình được lưu lại, dùng cho mọi mã QR sau này</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 302</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
           <t>BC-01</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Báo cáo</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Xuất Excel danh sách đơn hàng</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Khác</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Admin bấm xuất file Excel toàn bộ đơn hàng</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>File Excel tải về thành công, có dữ liệu bên trong</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>ĐẠT</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>5405 bytes</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>14/09/2026 15:11</t>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>5449 bytes</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add bulk select for orders: mark done/owed, or delete (super_admin only)
Same bulk-select pattern as the products and rooms pages. The route is
@admin_required since marking orders done/owed is routine admin work, but
the delete branch re-checks session.admin_role itself before touching
anything - same defense-in-depth pattern generate_bank_qr already used for
its set_default action - so bulk delete stays exclusively super_admin even
though it shares the endpoint. The delete button itself is also hidden
from the template for non-super-admins, matching the single-order delete
button already in place.

Verified live in a real browser plus 3 new CRUD test cases (DH-06/07/08)
- 48/48 passing.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test case/test_cases.xlsx
+++ b/Test case/test_cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1370,12 +1370,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>đơn 6-&gt;7, tồn kho 49-&gt;48</t>
+          <t>đơn 6-&gt;7, tồn kho 50-&gt;49</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1577,32 +1577,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>GH-01</t>
+          <t>DH-06</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Thêm vào giỏ hàng</t>
+          <t>Đánh dấu hàng loạt "đã xong" / "còn nợ"</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Khách thêm một sản phẩm vào giỏ hàng</t>
+          <t>Admin chọn nhiều đơn hàng cùng lúc rồi đánh dấu tất cả đã hoàn thành, sau đó chuyển lại thành còn nợ</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Sản phẩm xuất hiện trong giỏ với đúng số lượng</t>
+          <t>Tất cả đơn được chọn đổi đúng trạng thái, đơn không được chọn giữ nguyên</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -1610,10 +1610,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>o1=completed o2=completed o3 (untouched)=pending</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1623,32 +1627,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>GH-02</t>
+          <t>DH-07</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật số lượng trong giỏ</t>
+          <t>Xóa hàng loạt đơn hàng - Super Admin</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Khách đổi số lượng một sản phẩm đang có trong giỏ</t>
+          <t>Super Admin chọn nhiều đơn hàng rồi xóa cùng lúc</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Số lượng trong giỏ được cập nhật đúng</t>
+          <t>Tất cả đơn được chọn (và các dòng sản phẩm của chúng) bị xóa hẳn</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1656,10 +1660,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>o1 gone=True o2 gone=True items gone=True</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1669,17 +1677,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>GH-03</t>
+          <t>DH-08</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Giỏ hàng</t>
+          <t>Đơn hàng</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Xóa một món khỏi giỏ</t>
+          <t>Xóa hàng loạt đơn hàng - Admin thường (phải bị chặn)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1689,12 +1697,12 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Khách xóa một sản phẩm khỏi giỏ hàng</t>
+          <t>Tài khoản admin thường cố xóa hàng loạt đơn hàng</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Sản phẩm biến mất khỏi giỏ hàng</t>
+          <t>Bị từ chối, tất cả đơn hàng vẫn còn nguyên</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -1702,10 +1710,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>còn tồn tại=True</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1727,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>GH-04</t>
+          <t>GH-01</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1725,22 +1737,22 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Xóa nhiều món cùng lúc</t>
+          <t>Thêm vào giỏ hàng</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Khách tick chọn nhiều sản phẩm rồi xóa cùng lúc</t>
+          <t>Khách thêm một sản phẩm vào giỏ hàng</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Chỉ những sản phẩm được chọn bị xóa, các món khác vẫn còn</t>
+          <t>Sản phẩm xuất hiện trong giỏ với đúng số lượng</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -1748,14 +1760,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>gone=True kept=True</t>
-        </is>
-      </c>
+      <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1773,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CN-01</t>
+          <t>GH-02</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Công nợ</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Thanh toán một đơn nợ</t>
+          <t>Cập nhật số lượng trong giỏ</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1785,12 +1793,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Super Admin xác nhận một đơn còn nợ đã được trả</t>
+          <t>Khách đổi số lượng một sản phẩm đang có trong giỏ</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái đơn chuyển thành hoàn thành</t>
+          <t>Số lượng trong giỏ được cập nhật đúng</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -1801,7 +1809,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1811,32 +1819,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>CN-02</t>
+          <t>GH-03</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Công nợ</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Thanh toán nhiều đơn nợ cùng lúc</t>
+          <t>Xóa một món khỏi giỏ</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Super Admin chọn nhiều đơn nợ và xác nhận trả cùng lúc</t>
+          <t>Khách xóa một sản phẩm khỏi giỏ hàng</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Tất cả các đơn được chọn chuyển thành hoàn thành</t>
+          <t>Sản phẩm biến mất khỏi giỏ hàng</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1847,7 +1855,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1857,32 +1865,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>TK-01</t>
+          <t>GH-04</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Giỏ hàng</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Thêm tài khoản admin mới</t>
+          <t>Xóa nhiều món cùng lúc</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Super Admin tạo một tài khoản admin mới</t>
+          <t>Khách tick chọn nhiều sản phẩm rồi xóa cùng lúc</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản mới xuất hiện trong danh sách, đăng nhập được</t>
+          <t>Chỉ những sản phẩm được chọn bị xóa, các món khác vẫn còn</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -1892,12 +1900,12 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>2 -&gt; 3</t>
+          <t>gone=True kept=True</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1907,17 +1915,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>TK-02</t>
+          <t>CN-01</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Công nợ</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Đổi vai trò admin</t>
+          <t>Thanh toán một đơn nợ</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1927,12 +1935,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đổi vai trò một tài khoản admin thành super_admin</t>
+          <t>Super Admin xác nhận một đơn còn nợ đã được trả</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Vai trò được cập nhật đúng</t>
+          <t>Trạng thái đơn chuyển thành hoàn thành</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -1943,7 +1951,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1953,17 +1961,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>TK-03</t>
+          <t>CN-02</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản</t>
+          <t>Công nợ</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Đặt lại mật khẩu admin</t>
+          <t>Thanh toán nhiều đơn nợ cùng lúc</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1973,12 +1981,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đặt mật khẩu mới cho một tài khoản admin khác</t>
+          <t>Super Admin chọn nhiều đơn nợ và xác nhận trả cùng lúc</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản đó đăng nhập được bằng mật khẩu mới</t>
+          <t>Tất cả các đơn được chọn chuyển thành hoàn thành</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1989,7 +1997,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -1999,7 +2007,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>TK-04</t>
+          <t>TK-01</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2009,22 +2017,22 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Đặt lại mật khẩu khách hàng</t>
+          <t>Thêm tài khoản admin mới</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đặt mật khẩu mới cho một tài khoản khách hàng</t>
+          <t>Super Admin tạo một tài khoản admin mới</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản khách hàng đăng nhập được bằng mật khẩu mới</t>
+          <t>Tài khoản mới xuất hiện trong danh sách, đăng nhập được</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -2032,10 +2040,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2 -&gt; 3</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2057,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>TK-05</t>
+          <t>TK-02</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2055,22 +2067,22 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Xóa tài khoản admin</t>
+          <t>Đổi vai trò admin</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Super Admin xóa một tài khoản admin (không phải Super Admin cuối cùng)</t>
+          <t>Super Admin đổi vai trò một tài khoản admin thành super_admin</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản bị xóa hẳn, không đăng nhập được nữa</t>
+          <t>Vai trò được cập nhật đúng</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -2081,7 +2093,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2103,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>TK-06</t>
+          <t>TK-03</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2101,22 +2113,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Không cho xóa Super Admin cuối cùng</t>
+          <t>Đặt lại mật khẩu admin</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Xóa</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Super Admin cố xóa chính Super Admin cuối cùng còn lại trong hệ thống</t>
+          <t>Super Admin đặt mật khẩu mới cho một tài khoản admin khác</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Bị từ chối, luôn còn ít nhất một Super Admin</t>
+          <t>Tài khoản đó đăng nhập được bằng mật khẩu mới</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2124,14 +2136,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>còn tồn tại=True</t>
-        </is>
-      </c>
+      <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2149,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>TK-07</t>
+          <t>TK-04</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2151,7 +2159,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Bật/tắt quyền Manager</t>
+          <t>Đặt lại mật khẩu khách hàng</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2161,12 +2169,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Super Admin cấp rồi thu hồi quyền Manager cho một khách hàng</t>
+          <t>Super Admin đặt mật khẩu mới cho một tài khoản khách hàng</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Vai trò khách hàng đổi qua lại đúng giữa customer và manager</t>
+          <t>Tài khoản khách hàng đăng nhập được bằng mật khẩu mới</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -2174,14 +2182,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>promoted=True back=True</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2195,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>TK-08</t>
+          <t>TK-05</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2201,22 +2205,22 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Đăng ký tài khoản khách hàng</t>
+          <t>Xóa tài khoản admin</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Khách tự đăng ký tài khoản mới trên trang web</t>
+          <t>Super Admin xóa một tài khoản admin (không phải Super Admin cuối cùng)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản khách hàng mới được tạo, đăng nhập được ngay</t>
+          <t>Tài khoản bị xóa hẳn, không đăng nhập được nữa</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -2224,14 +2228,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>0 -&gt; 1</t>
-        </is>
-      </c>
+      <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2241,32 +2241,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>XT-01</t>
+          <t>TK-06</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập admin đúng mật khẩu</t>
+          <t>Không cho xóa Super Admin cuối cùng</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Xóa</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập với tài khoản/mật khẩu admin đúng</t>
+          <t>Super Admin cố xóa chính Super Admin cuối cùng còn lại trong hệ thống</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập thành công, vào được trang quản trị</t>
+          <t>Bị từ chối, luôn còn ít nhất một Super Admin</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2274,10 +2274,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>còn tồn tại=True</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2287,32 +2291,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>XT-02</t>
+          <t>TK-07</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập admin sai mật khẩu</t>
+          <t>Bật/tắt quyền Manager</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập với mật khẩu sai</t>
+          <t>Super Admin cấp rồi thu hồi quyền Manager cho một khách hàng</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Bị từ chối, không vào được trang quản trị</t>
+          <t>Vai trò khách hàng đổi qua lại đúng giữa customer và manager</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2322,12 +2326,12 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302</t>
+          <t>promoted=True back=True</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2337,32 +2341,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>XT-03</t>
+          <t>TK-08</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Xác thực</t>
+          <t>Tài khoản</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Admin tự đổi mật khẩu</t>
+          <t>Đăng ký tài khoản khách hàng</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Thêm</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Admin đang đăng nhập tự đổi mật khẩu của chính mình</t>
+          <t>Khách tự đăng ký tài khoản mới trên trang web</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập lại bằng mật khẩu mới thành công</t>
+          <t>Tài khoản khách hàng mới được tạo, đăng nhập được ngay</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2370,10 +2374,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>0 -&gt; 1</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2391,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>XT-04</t>
+          <t>XT-01</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2393,7 +2401,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập khách hàng</t>
+          <t>Đăng nhập admin đúng mật khẩu</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2403,12 +2411,12 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Khách đăng nhập bằng tài khoản đã đăng ký</t>
+          <t>Đăng nhập với tài khoản/mật khẩu admin đúng</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập thành công</t>
+          <t>Đăng nhập thành công, vào được trang quản trị</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -2416,14 +2424,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>HTTP 302</t>
-        </is>
-      </c>
+      <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2437,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>XT-05</t>
+          <t>XT-02</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2443,7 +2447,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Đăng xuất khách hàng</t>
+          <t>Đăng nhập admin sai mật khẩu</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2453,12 +2457,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Khách đã đăng nhập bấm đăng xuất</t>
+          <t>Đăng nhập với mật khẩu sai</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Phiên đăng nhập kết thúc</t>
+          <t>Bị từ chối, không vào được trang quản trị</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -2466,10 +2470,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 302</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2479,32 +2487,32 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>QR-01</t>
+          <t>XT-03</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>QR / Thanh toán</t>
+          <t>Xác thực</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Tạo mã QR tuỳ ý</t>
+          <t>Admin tự đổi mật khẩu</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Sửa</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Admin tạo một mã QR từ nội dung bất kỳ</t>
+          <t>Admin đang đăng nhập tự đổi mật khẩu của chính mình</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Ảnh mã QR được sinh ra thành công</t>
+          <t>Đăng nhập lại bằng mật khẩu mới thành công</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2515,7 +2523,7 @@
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2525,32 +2533,32 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>QR-02</t>
+          <t>XT-04</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>QR / Thanh toán</t>
+          <t>Xác thực</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Tạo mã QR chuyển khoản ngân hàng</t>
+          <t>Đăng nhập khách hàng</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Thêm</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Admin tạo mã QR chuyển khoản với số tiền và nội dung</t>
+          <t>Khách đăng nhập bằng tài khoản đã đăng ký</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Ảnh mã QR VietQR được sinh ra thành công</t>
+          <t>Đăng nhập thành công</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2558,10 +2566,14 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 302</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2571,32 +2583,32 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>QR-03</t>
+          <t>XT-05</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>QR / Thanh toán</t>
+          <t>Xác thực</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Đặt tài khoản nhận tiền mặc định</t>
+          <t>Đăng xuất khách hàng</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Sửa</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Super Admin đặt một tài khoản ngân hàng làm tài khoản nhận tiền mặc định của quán</t>
+          <t>Khách đã đăng nhập bấm đăng xuất</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Cấu hình được lưu lại, dùng cho mọi mã QR sau này</t>
+          <t>Phiên đăng nhập kết thúc</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -2604,14 +2616,10 @@
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>HTTP 302</t>
-        </is>
-      </c>
+      <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>14/09/2026 15:27</t>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>
@@ -2621,47 +2629,189 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
+          <t>QR-01</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>QR / Thanh toán</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Tạo mã QR tuỳ ý</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Thêm</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Admin tạo một mã QR từ nội dung bất kỳ</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh mã QR được sinh ra thành công</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>QR-02</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>QR / Thanh toán</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Tạo mã QR chuyển khoản ngân hàng</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Thêm</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Admin tạo mã QR chuyển khoản với số tiền và nội dung</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh mã QR VietQR được sinh ra thành công</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>QR-03</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>QR / Thanh toán</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Đặt tài khoản nhận tiền mặc định</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Sửa</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Super Admin đặt một tài khoản ngân hàng làm tài khoản nhận tiền mặc định của quán</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình được lưu lại, dùng cho mọi mã QR sau này</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 302</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
           <t>BC-01</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Báo cáo</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Xuất Excel danh sách đơn hàng</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Khác</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Admin bấm xuất file Excel toàn bộ đơn hàng</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>File Excel tải về thành công, có dữ liệu bên trong</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>ĐẠT</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>5449 bytes</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>14/09/2026 15:27</t>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>5518 bytes</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026 15:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix leftover "Coffee Vibes" placeholder in the order-success message
Found by actually placing a real order end-to-end as a customer would -
the success banner after checkout still said "Cảm ơn bạn đã mua hàng tại
Coffee Vibes", a leftover from whatever demo template this project started
from. Every customer who ever completed an order saw this. Now says
"Cô Bông Cát Lái" like everywhere else on the site.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test case/test_cases.xlsx
+++ b/Test case/test_cases.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1370,12 +1370,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>đơn 7-&gt;8, tồn kho 53-&gt;52</t>
+          <t>đơn 7-&gt;8, tồn kho 55-&gt;54</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2293,7 +2293,7 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -3106,12 +3106,12 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>all có cả 2=True, lọc nợ chỉ còn={'Người Nhận Hộ', 'QA Export Debt', 'QA Bulk Order 3 (untouched)', 'Nguyễn Văn Test', 'Nguyễn Văn An', 'Kiem tra dinh dang'}</t>
+          <t>all có cả 2=True, lọc nợ chỉ còn={'Người Nhận Hộ', 'QA Bulk Order 3 (untouched)', 'QA Export Debt', 'Nguyễn Văn Test', 'Nguyễn Văn An', 'Kiem tra dinh dang'}</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>15/09/2026 15:05</t>
+          <t>15/09/2026 16:55</t>
         </is>
       </c>
     </row>

</xml_diff>